<commit_message>
feat: add IPO application management module, expand trading strategies documentation, and integrate Telegram notification diagnostics into dashboard
</commit_message>
<xml_diff>
--- a/allotted_holdings.xlsx
+++ b/allotted_holdings.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CapitalFund1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5BB23AA-8CD6-44A9-87D6-96040B8AF06E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00040921-B672-4939-A848-27F62AA86372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="2340" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1" sheetId="1" r:id="rId1"/>
+    <sheet name="2" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="12">
   <si>
     <t>security_name</t>
   </si>
@@ -649,4 +650,211 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CFACDDA-46F8-4347-A644-C0B466288384}">
+  <dimension ref="A1:AJ24"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.88671875" customWidth="1"/>
+    <col min="3" max="3" width="13.88671875" customWidth="1"/>
+    <col min="4" max="4" width="16.5546875" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" customWidth="1"/>
+    <col min="8" max="8" width="23.5546875" customWidth="1"/>
+    <col min="9" max="9" width="26.33203125" customWidth="1"/>
+    <col min="10" max="10" width="21.88671875" customWidth="1"/>
+    <col min="11" max="11" width="22.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:36" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2">
+        <v>200</v>
+      </c>
+      <c r="C2">
+        <v>400</v>
+      </c>
+      <c r="D2">
+        <v>500</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>5</v>
+      </c>
+      <c r="X2">
+        <v>1</v>
+      </c>
+      <c r="Y2">
+        <v>0</v>
+      </c>
+      <c r="Z2">
+        <v>0</v>
+      </c>
+      <c r="AA2">
+        <v>0</v>
+      </c>
+      <c r="AC2">
+        <v>0</v>
+      </c>
+      <c r="AJ2">
+        <v>12.157500000000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="H3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="H4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="H5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="H6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="H7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="H8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="H9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="H10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="H11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="H12">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="H13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="H14">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="H15">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="H16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H19">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H20">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H21">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H22">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H23">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H24">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>